<commit_message>
Add BCM and Dynamo (vLLM) connectors, six DCGM prompts (G17–G22)
New truth sources (truth/bcm.py: BCM REST over mTLS; truth/dynamo.py: vLLM /metrics), checks (grading/bcm_dynamo.py; gpu.py + 4 DCGM checks), sheet data/bcm_dynamo_prompts.xlsx (B01–B06, V01–V07) and G17–G22 in gpu_prompts.xlsx. runner: <MODEL> placeholder. chat/policy: follow-up detection matches curly apostrophes and 'could you tell me'; SLA questions answered 'TTFT SLA of 500 ms'. pytest.ini -n 8. Existing grading unchanged. Self-tests 190 -> 261.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gpu_prompts.xlsx
+++ b/data/gpu_prompts.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,188 @@
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Prometheus: slices = firing alerts per severity; with no alerts NCP must say so and draw no chart. DCGM: NA only if NCP says not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Show GPU utilization.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>gpu_util</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>dcgm</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Dev's sheet 2026-10-14 (DCGM). Every GPU ±GPU_UTIL_TOL of a read taken while NCP answered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>G18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>List every GPU with its host and card model.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>gpu_inventory</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>dcgm</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Every GPU (host + index) with its model (A6000, V100, PRO 6000 … count); another GPU's model = FAIL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>G19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Which GPU is running hottest right now?</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>gpu_hottest</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>dcgm</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Same check as G10 (other wording). First GPU named (host + index) is the hottest, ties ±TEMP_TOL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>G20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Show framebuffer memory used, free and reserved for each GPU.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>gpu_framebuffer</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>dcgm</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>DCGM_FI_DEV_FB_USED / FREE / RESERVED per GPU, MiB (GiB / GB × 1024), ±FB_TOL % (default 10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>G21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Show XID errors for all GPUs over the last 7 days.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>gpu_xid</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>dcgm</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Param = hours. max_over_time(XID) per GPU: GPUs with an XID named, none claimed for a GPU at 0; 'no XID' when none. hgx-su00-v100 has no XID series: not graded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>G22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Are any GPUs currently clock throttled?</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>throttling</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>dcgm</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Same check as G08 (other wording): no throttling series — NCP's per-GPU values vs the reads at its tool-call time; NA on 'not available'.</t>
         </is>
       </c>
     </row>
@@ -995,7 +1177,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hours of the time window (G03–G05, G15), the idle threshold % (G12), the temperature limit °C (G14).</t>
+          <t>Hours of the time window (G03–G05, G15, G21), the idle threshold % (G12), the temperature limit °C (G14).</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1201,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Comma list of connectors (prometheus, dcgm). Blank = both.</t>
+          <t>Comma list of connectors (prometheus, dcgm). Blank = both. G17–G22: dcgm only (Dev's 2026-10-14 sheet).</t>
         </is>
       </c>
     </row>

</xml_diff>